<commit_message>
fix : 소비 기물 item의 effectType 수정
* 테이블의 effectType 값을 Enums.cs 파일에 입력된 값과 같도록 변경
</commit_message>
<xml_diff>
--- a/Assets/Resources/Excel/Item.xlsx
+++ b/Assets/Resources/Excel/Item.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24334"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHubProjects\UnityProject_LucidDiver\Assets\Resources\Excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Woo_260126\UnityProject_LucidDiver\Assets\Resources\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AE3BDE0-26AB-47EA-A56C-C554BCC06709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{622F18E1-3D01-45D5-A6EF-F26F7AF069A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2145" yWindow="1185" windowWidth="21480" windowHeight="13380" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,8 +27,6 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -140,9 +138,6 @@
     <t>self</t>
   </si>
   <si>
-    <t>health_recover_inst</t>
-  </si>
-  <si>
     <t>이상한 사탕</t>
   </si>
   <si>
@@ -150,9 +145,6 @@
   </si>
   <si>
     <t>Image_302_WeirdCandy</t>
-  </si>
-  <si>
-    <t>mana_recover_inst</t>
   </si>
   <si>
     <t>기억 조각</t>
@@ -179,6 +171,14 @@
   </si>
   <si>
     <t>epic</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>healHP</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>healMP</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -245,9 +245,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -285,7 +285,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -391,7 +391,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -533,7 +533,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -647,7 +647,7 @@
         <v>1</v>
       </c>
       <c r="F2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
         <v>26</v>
@@ -706,7 +706,7 @@
         <v>32</v>
       </c>
       <c r="S3" t="s">
-        <v>33</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.3">
@@ -714,10 +714,10 @@
         <v>302</v>
       </c>
       <c r="B4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C4" t="s">
         <v>34</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
       </c>
       <c r="D4" t="s">
         <v>29</v>
@@ -726,10 +726,10 @@
         <v>5</v>
       </c>
       <c r="F4" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="N4" t="s">
         <v>31</v>
@@ -747,7 +747,7 @@
         <v>32</v>
       </c>
       <c r="S4" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.3">
@@ -755,25 +755,25 @@
         <v>401</v>
       </c>
       <c r="B5" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
         <v>38</v>
-      </c>
-      <c r="C5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D5" t="s">
-        <v>40</v>
       </c>
       <c r="E5">
         <v>10</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="T5" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="U5">
         <v>0</v>
@@ -785,5 +785,6 @@
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>